<commit_message>
Vzorová data: Provize 5 000, Produkce 30 000
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/vzorova-data.xlsx
+++ b/vzorova-data.xlsx
@@ -1,88 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11027"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/danielvojik/Downloads/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9716DD0A-39C7-E143-84DF-189E919309F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="2060" yWindow="1280" windowWidth="27840" windowHeight="16740" xr2:uid="{AEDDC349-F607-AF49-A210-F547A0F6B1D4}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2060" yWindow="1280" windowWidth="27840" windowHeight="16740" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="List1" sheetId="1" r:id="rId1"/>
+    <sheet name="List1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="181029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Jméno</t>
-  </si>
-  <si>
-    <t>Ivana Vojíková</t>
-  </si>
-  <si>
-    <t>Provize</t>
-  </si>
-  <si>
-    <t>eKoruny</t>
-  </si>
-  <si>
-    <t>Produkce</t>
-  </si>
-  <si>
-    <t>Smlouvy</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="6" formatCode="#,##0\ &quot;Kč&quot;;[Red]\-#,##0\ &quot;Kč&quot;"/>
+    <numFmt numFmtId="164" formatCode="#,##0\ &quot;Kč&quot;;[Red]\-#,##0\ &quot;Kč&quot;"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
+      <name val="Aptos Narrow"/>
+      <charset val="238"/>
+      <family val="2"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Aptos Narrow"/>
+      <b val="1"/>
+      <color theme="1"/>
       <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -100,24 +55,84 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+  <cellXfs count="4">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -437,49 +452,65 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5AB0EDE-D7CE-CD47-BB04-6981D4CE6311}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
+    <col width="18" bestFit="1" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="2" t="s">
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Jméno</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Provize</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>eKoruny</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Produkce</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Smlouvy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ivana Vojíková</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="C2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E2" t="n">
         <v>4</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>5000</v>
-      </c>
-      <c r="C2">
-        <v>100</v>
-      </c>
-      <c r="D2" s="1">
-        <v>30000</v>
-      </c>
-      <c r="E2">
-        <v>4</v>
-      </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="3" t="n"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <pageMargins left="0.7" right="0.7" top="0.787401575" bottom="0.787401575" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>